<commit_message>
bakced up some Tikhonov reg stuff
</commit_message>
<xml_diff>
--- a/Notebooks/TestDataLots.xlsx
+++ b/Notebooks/TestDataLots.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\University_Materials\2024\P4P\p4p-geothermalML\Notebooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9386691-A361-43DC-9826-EFA4B191E8CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76A72DD2-E6C3-4144-B6DF-C9F3E0F2FF10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TotalMassFlow" sheetId="1" r:id="rId1"/>
@@ -3328,10 +3328,10 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="B20">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="C20">
         <v>0</v>
@@ -3368,7 +3368,7 @@
         <v>1</v>
       </c>
       <c r="C22">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="D22">
         <v>0</v>
@@ -3405,7 +3405,7 @@
         <v>1</v>
       </c>
       <c r="D24">
-        <v>1</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="E24">
         <v>0</v>
@@ -3422,7 +3422,7 @@
         <v>1</v>
       </c>
       <c r="D25">
-        <v>1</v>
+        <v>0.82</v>
       </c>
       <c r="E25">
         <v>0</v>
@@ -3510,7 +3510,7 @@
         <v>1</v>
       </c>
       <c r="E30">
-        <v>1</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>